<commit_message>
update popd case study
</commit_message>
<xml_diff>
--- a/gcmc_data_codes/Case of population density study/Case of population density study.xlsx
+++ b/gcmc_data_codes/Case of population density study/Case of population density study.xlsx
@@ -392,10 +392,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.6186578798185941</v>
+        <v>0.5866800103305785</v>
       </c>
       <c r="D2">
-        <v>0.0006192749108928587</v>
+        <v>0.01102583290842787</v>
       </c>
     </row>
     <row r="3">
@@ -410,10 +410,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.1063633786848073</v>
+        <v>0.07818956611570248</v>
       </c>
       <c r="D3">
-        <v>2.155995784578711E-74</v>
+        <v>2.817486482679664E-119</v>
       </c>
     </row>
     <row r="4">
@@ -428,10 +428,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.3006306689342403</v>
+        <v>0.2730178202479339</v>
       </c>
       <c r="D4">
-        <v>1.757118450130801E-09</v>
+        <v>3.996458043291421E-13</v>
       </c>
     </row>
     <row r="5">
@@ -446,10 +446,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.09279336734693877</v>
+        <v>0.07644628099173553</v>
       </c>
       <c r="D5">
-        <v>7.74111461817066E-95</v>
+        <v>1.466164569681461E-125</v>
       </c>
     </row>
     <row r="6">
@@ -464,10 +464,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.2424178004535147</v>
+        <v>0.2188468491735537</v>
       </c>
       <c r="D6">
-        <v>1.674870268848038E-16</v>
+        <v>6.996948658564489E-22</v>
       </c>
     </row>
     <row r="7">
@@ -482,10 +482,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.5001771541950113</v>
+        <v>0.4734956095041322</v>
       </c>
       <c r="D7">
-        <v>0.9961253644644774</v>
+        <v>0.4541298647699026</v>
       </c>
     </row>
   </sheetData>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.7291112340047295</v>
+        <v>0.7062124050712434</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.4049899717392104</v>
+        <v>0.4066616656061571</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.7242901714077293</v>
+        <v>0.7002693431487101</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.4292317231265871</v>
+        <v>0.4378726106424903</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.9167751824652264</v>
+        <v>0.9164397234774496</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.9279989762529879</v>
+        <v>0.9276983216868078</v>
       </c>
       <c r="D7">
         <v>0</v>

</xml_diff>